<commit_message>
Completed cleaning the Nebula_Galaxy data.
Next: Moving onto RB
</commit_message>
<xml_diff>
--- a/SWTest/Outputs/Finalists/DEET_Analysis_Final.xlsx
+++ b/SWTest/Outputs/Finalists/DEET_Analysis_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\Finalists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127AD1CD-63B1-4DDC-902D-044BA49B01BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F131990-A9E9-44BF-B658-DC2F707E90CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="4575" windowWidth="16410" windowHeight="16815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1301,8 +1301,8 @@
     <col min="4" max="5" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="59.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="59.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -1334,10 +1334,10 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>9</v>
@@ -1380,7 +1380,7 @@
       <c r="G2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H2" t="s">
         <v>21</v>
       </c>
       <c r="J2" t="s">
@@ -1415,7 +1415,7 @@
       <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="I3" t="s">
+      <c r="H3" t="s">
         <v>21</v>
       </c>
       <c r="K3" t="s">
@@ -1453,7 +1453,7 @@
       <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="I4" t="s">
+      <c r="H4" t="s">
         <v>30</v>
       </c>
       <c r="K4" t="s">
@@ -1488,7 +1488,7 @@
       <c r="F5" t="s">
         <v>19</v>
       </c>
-      <c r="I5" t="s">
+      <c r="H5" t="s">
         <v>30</v>
       </c>
       <c r="J5" t="s">
@@ -1523,7 +1523,7 @@
       <c r="F6" t="s">
         <v>19</v>
       </c>
-      <c r="I6" t="s">
+      <c r="H6" t="s">
         <v>30</v>
       </c>
       <c r="J6" t="s">
@@ -1558,7 +1558,7 @@
       <c r="F7" t="s">
         <v>19</v>
       </c>
-      <c r="I7" t="s">
+      <c r="H7" t="s">
         <v>21</v>
       </c>
       <c r="J7" t="s">
@@ -1593,7 +1593,7 @@
       <c r="F8" t="s">
         <v>19</v>
       </c>
-      <c r="I8" t="s">
+      <c r="H8" t="s">
         <v>21</v>
       </c>
       <c r="J8" t="s">
@@ -1628,7 +1628,7 @@
       <c r="F9" t="s">
         <v>19</v>
       </c>
-      <c r="I9" t="s">
+      <c r="H9" t="s">
         <v>30</v>
       </c>
       <c r="J9" t="s">
@@ -1663,7 +1663,7 @@
       <c r="F10" t="s">
         <v>19</v>
       </c>
-      <c r="I10" t="s">
+      <c r="H10" t="s">
         <v>30</v>
       </c>
       <c r="J10" t="s">
@@ -1698,7 +1698,7 @@
       <c r="F11" t="s">
         <v>19</v>
       </c>
-      <c r="I11" t="s">
+      <c r="H11" t="s">
         <v>21</v>
       </c>
       <c r="J11" t="s">
@@ -1733,7 +1733,7 @@
       <c r="F12" t="s">
         <v>19</v>
       </c>
-      <c r="I12" t="s">
+      <c r="H12" t="s">
         <v>21</v>
       </c>
       <c r="J12" t="s">
@@ -1768,7 +1768,7 @@
       <c r="F13" t="s">
         <v>19</v>
       </c>
-      <c r="I13" t="s">
+      <c r="H13" t="s">
         <v>21</v>
       </c>
       <c r="J13" t="s">
@@ -1803,7 +1803,7 @@
       <c r="F14" t="s">
         <v>19</v>
       </c>
-      <c r="I14" t="s">
+      <c r="H14" t="s">
         <v>21</v>
       </c>
       <c r="J14" t="s">
@@ -1841,7 +1841,7 @@
       <c r="F15" t="s">
         <v>19</v>
       </c>
-      <c r="I15" t="s">
+      <c r="H15" t="s">
         <v>21</v>
       </c>
       <c r="J15" t="s">
@@ -1879,7 +1879,7 @@
       <c r="F16" t="s">
         <v>19</v>
       </c>
-      <c r="I16" t="s">
+      <c r="H16" t="s">
         <v>21</v>
       </c>
       <c r="J16" t="s">
@@ -1914,7 +1914,7 @@
       <c r="F17" t="s">
         <v>19</v>
       </c>
-      <c r="I17" t="s">
+      <c r="H17" t="s">
         <v>21</v>
       </c>
       <c r="J17" t="s">
@@ -1949,7 +1949,7 @@
       <c r="F18" t="s">
         <v>19</v>
       </c>
-      <c r="I18" t="s">
+      <c r="H18" t="s">
         <v>21</v>
       </c>
       <c r="J18" t="s">
@@ -1984,7 +1984,7 @@
       <c r="F19" t="s">
         <v>19</v>
       </c>
-      <c r="I19" t="s">
+      <c r="H19" t="s">
         <v>77</v>
       </c>
       <c r="J19" t="s">
@@ -2025,7 +2025,7 @@
       <c r="G20" t="s">
         <v>20</v>
       </c>
-      <c r="I20" t="s">
+      <c r="H20" t="s">
         <v>21</v>
       </c>
       <c r="J20" t="s">
@@ -2066,7 +2066,7 @@
       <c r="G21" t="s">
         <v>20</v>
       </c>
-      <c r="I21" t="s">
+      <c r="H21" t="s">
         <v>21</v>
       </c>
       <c r="J21" t="s">
@@ -2107,7 +2107,7 @@
       <c r="G22" t="s">
         <v>20</v>
       </c>
-      <c r="I22" t="s">
+      <c r="H22" t="s">
         <v>77</v>
       </c>
       <c r="J22" t="s">
@@ -2148,7 +2148,7 @@
       <c r="G23" t="s">
         <v>20</v>
       </c>
-      <c r="I23" t="s">
+      <c r="H23" t="s">
         <v>21</v>
       </c>
       <c r="K23" t="s">
@@ -2180,7 +2180,7 @@
       <c r="F24" t="s">
         <v>19</v>
       </c>
-      <c r="I24" t="s">
+      <c r="H24" t="s">
         <v>30</v>
       </c>
       <c r="K24" t="s">
@@ -2218,7 +2218,7 @@
       <c r="F25" t="s">
         <v>19</v>
       </c>
-      <c r="I25" t="s">
+      <c r="H25" t="s">
         <v>30</v>
       </c>
       <c r="K25" t="s">
@@ -2256,7 +2256,7 @@
       <c r="F26" t="s">
         <v>19</v>
       </c>
-      <c r="I26" t="s">
+      <c r="H26" t="s">
         <v>30</v>
       </c>
       <c r="K26" t="s">
@@ -2294,7 +2294,7 @@
       <c r="F27" t="s">
         <v>19</v>
       </c>
-      <c r="I27" t="s">
+      <c r="H27" t="s">
         <v>30</v>
       </c>
       <c r="K27" t="s">
@@ -2332,7 +2332,7 @@
       <c r="F28" t="s">
         <v>19</v>
       </c>
-      <c r="I28" t="s">
+      <c r="H28" t="s">
         <v>30</v>
       </c>
       <c r="K28" t="s">
@@ -2370,7 +2370,7 @@
       <c r="F29" t="s">
         <v>19</v>
       </c>
-      <c r="I29" t="s">
+      <c r="H29" t="s">
         <v>30</v>
       </c>
       <c r="J29" t="s">
@@ -2405,7 +2405,7 @@
       <c r="F30" t="s">
         <v>19</v>
       </c>
-      <c r="I30" t="s">
+      <c r="H30" t="s">
         <v>30</v>
       </c>
       <c r="J30" t="s">
@@ -2440,7 +2440,7 @@
       <c r="F31" t="s">
         <v>19</v>
       </c>
-      <c r="I31" t="s">
+      <c r="H31" t="s">
         <v>21</v>
       </c>
       <c r="J31" t="s">
@@ -2481,7 +2481,7 @@
       <c r="F32" t="s">
         <v>19</v>
       </c>
-      <c r="I32" t="s">
+      <c r="H32" t="s">
         <v>21</v>
       </c>
       <c r="J32" t="s">
@@ -2522,7 +2522,7 @@
       <c r="F33" t="s">
         <v>19</v>
       </c>
-      <c r="I33" t="s">
+      <c r="H33" t="s">
         <v>21</v>
       </c>
       <c r="J33" t="s">
@@ -2557,7 +2557,7 @@
       <c r="F34" t="s">
         <v>19</v>
       </c>
-      <c r="I34" t="s">
+      <c r="H34" t="s">
         <v>77</v>
       </c>
       <c r="J34" t="s">
@@ -2598,7 +2598,7 @@
       <c r="G35" t="s">
         <v>126</v>
       </c>
-      <c r="I35" t="s">
+      <c r="H35" t="s">
         <v>21</v>
       </c>
       <c r="J35" t="s">
@@ -2639,7 +2639,7 @@
       <c r="F36" t="s">
         <v>19</v>
       </c>
-      <c r="I36" t="s">
+      <c r="H36" t="s">
         <v>30</v>
       </c>
       <c r="J36" t="s">
@@ -2677,7 +2677,7 @@
       <c r="F37" t="s">
         <v>19</v>
       </c>
-      <c r="I37" t="s">
+      <c r="H37" t="s">
         <v>21</v>
       </c>
       <c r="K37" t="s">
@@ -2715,7 +2715,7 @@
       <c r="G38" t="s">
         <v>139</v>
       </c>
-      <c r="I38" t="s">
+      <c r="H38" t="s">
         <v>30</v>
       </c>
       <c r="J38" t="s">
@@ -2756,7 +2756,7 @@
       <c r="F39" t="s">
         <v>19</v>
       </c>
-      <c r="I39" t="s">
+      <c r="H39" t="s">
         <v>30</v>
       </c>
       <c r="K39" t="s">
@@ -2794,7 +2794,7 @@
       <c r="F40" t="s">
         <v>19</v>
       </c>
-      <c r="I40" t="s">
+      <c r="H40" t="s">
         <v>30</v>
       </c>
       <c r="J40" t="s">
@@ -2832,7 +2832,7 @@
       <c r="F41" t="s">
         <v>19</v>
       </c>
-      <c r="I41" t="s">
+      <c r="H41" t="s">
         <v>21</v>
       </c>
       <c r="K41" t="s">
@@ -2867,7 +2867,7 @@
       <c r="F42" t="s">
         <v>19</v>
       </c>
-      <c r="I42" t="s">
+      <c r="H42" t="s">
         <v>21</v>
       </c>
       <c r="K42" t="s">
@@ -2902,7 +2902,7 @@
       <c r="F43" t="s">
         <v>19</v>
       </c>
-      <c r="I43" t="s">
+      <c r="H43" t="s">
         <v>21</v>
       </c>
       <c r="K43" t="s">
@@ -2937,7 +2937,7 @@
       <c r="F44" t="s">
         <v>19</v>
       </c>
-      <c r="I44" t="s">
+      <c r="H44" t="s">
         <v>21</v>
       </c>
       <c r="K44" t="s">
@@ -2972,7 +2972,7 @@
       <c r="F45" t="s">
         <v>18</v>
       </c>
-      <c r="I45" t="s">
+      <c r="H45" t="s">
         <v>21</v>
       </c>
       <c r="K45" t="s">
@@ -3004,7 +3004,7 @@
       <c r="F46" t="s">
         <v>18</v>
       </c>
-      <c r="I46" t="s">
+      <c r="H46" t="s">
         <v>21</v>
       </c>
       <c r="K46" t="s">
@@ -3036,7 +3036,7 @@
       <c r="F47" t="s">
         <v>18</v>
       </c>
-      <c r="I47" t="s">
+      <c r="H47" t="s">
         <v>21</v>
       </c>
       <c r="K47" t="s">
@@ -3068,7 +3068,7 @@
       <c r="F48" t="s">
         <v>18</v>
       </c>
-      <c r="I48" t="s">
+      <c r="H48" t="s">
         <v>21</v>
       </c>
       <c r="K48" t="s">
@@ -3100,7 +3100,7 @@
       <c r="F49" t="s">
         <v>19</v>
       </c>
-      <c r="I49" t="s">
+      <c r="H49" t="s">
         <v>21</v>
       </c>
       <c r="K49" t="s">
@@ -3132,7 +3132,7 @@
       <c r="F50" t="s">
         <v>19</v>
       </c>
-      <c r="I50" t="s">
+      <c r="H50" t="s">
         <v>30</v>
       </c>
       <c r="J50" t="s">
@@ -3170,7 +3170,7 @@
       <c r="F51" t="s">
         <v>19</v>
       </c>
-      <c r="I51" t="s">
+      <c r="H51" t="s">
         <v>21</v>
       </c>
       <c r="K51" t="s">
@@ -3237,7 +3237,7 @@
       <c r="F53" t="s">
         <v>19</v>
       </c>
-      <c r="I53" t="s">
+      <c r="H53" t="s">
         <v>21</v>
       </c>
       <c r="J53" t="s">
@@ -3272,7 +3272,7 @@
       <c r="F54" t="s">
         <v>19</v>
       </c>
-      <c r="I54" t="s">
+      <c r="H54" t="s">
         <v>21</v>
       </c>
       <c r="K54" t="s">
@@ -3304,7 +3304,7 @@
       <c r="F55" t="s">
         <v>19</v>
       </c>
-      <c r="I55" t="s">
+      <c r="H55" t="s">
         <v>30</v>
       </c>
       <c r="J55" t="s">
@@ -3339,7 +3339,7 @@
       <c r="F56" t="s">
         <v>19</v>
       </c>
-      <c r="I56" t="s">
+      <c r="H56" t="s">
         <v>30</v>
       </c>
       <c r="J56" t="s">
@@ -3374,7 +3374,7 @@
       <c r="F57" t="s">
         <v>19</v>
       </c>
-      <c r="I57" t="s">
+      <c r="H57" t="s">
         <v>30</v>
       </c>
       <c r="J57" t="s">
@@ -3409,7 +3409,7 @@
       <c r="F58" t="s">
         <v>19</v>
       </c>
-      <c r="I58" t="s">
+      <c r="H58" t="s">
         <v>30</v>
       </c>
       <c r="J58" t="s">
@@ -3444,7 +3444,7 @@
       <c r="F59" t="s">
         <v>19</v>
       </c>
-      <c r="I59" t="s">
+      <c r="H59" t="s">
         <v>30</v>
       </c>
       <c r="K59" t="s">
@@ -3476,7 +3476,7 @@
       <c r="F60" t="s">
         <v>19</v>
       </c>
-      <c r="I60" t="s">
+      <c r="H60" t="s">
         <v>30</v>
       </c>
       <c r="J60" t="s">
@@ -3511,7 +3511,7 @@
       <c r="F61" t="s">
         <v>19</v>
       </c>
-      <c r="I61" t="s">
+      <c r="H61" t="s">
         <v>21</v>
       </c>
       <c r="J61" t="s">
@@ -3546,7 +3546,7 @@
       <c r="F62" t="s">
         <v>19</v>
       </c>
-      <c r="I62" t="s">
+      <c r="H62" t="s">
         <v>21</v>
       </c>
       <c r="J62" t="s">
@@ -3581,7 +3581,7 @@
       <c r="F63" t="s">
         <v>19</v>
       </c>
-      <c r="I63" t="s">
+      <c r="H63" t="s">
         <v>21</v>
       </c>
       <c r="K63" t="s">
@@ -3613,7 +3613,7 @@
       <c r="F64" t="s">
         <v>19</v>
       </c>
-      <c r="I64" t="s">
+      <c r="H64" t="s">
         <v>21</v>
       </c>
       <c r="K64" t="s">
@@ -3645,7 +3645,7 @@
       <c r="F65" t="s">
         <v>19</v>
       </c>
-      <c r="I65" t="s">
+      <c r="H65" t="s">
         <v>21</v>
       </c>
       <c r="K65" t="s">
@@ -3677,7 +3677,7 @@
       <c r="F66" t="s">
         <v>19</v>
       </c>
-      <c r="I66" t="s">
+      <c r="H66" t="s">
         <v>21</v>
       </c>
       <c r="K66" t="s">
@@ -3709,7 +3709,7 @@
       <c r="F67" t="s">
         <v>19</v>
       </c>
-      <c r="I67" t="s">
+      <c r="H67" t="s">
         <v>21</v>
       </c>
       <c r="J67" t="s">
@@ -3744,7 +3744,7 @@
       <c r="F68" t="s">
         <v>19</v>
       </c>
-      <c r="I68" t="s">
+      <c r="H68" t="s">
         <v>21</v>
       </c>
       <c r="J68" t="s">
@@ -3779,7 +3779,7 @@
       <c r="F69" t="s">
         <v>19</v>
       </c>
-      <c r="I69" t="s">
+      <c r="H69" t="s">
         <v>21</v>
       </c>
       <c r="J69" t="s">
@@ -3814,7 +3814,7 @@
       <c r="F70" t="s">
         <v>19</v>
       </c>
-      <c r="I70" t="s">
+      <c r="H70" t="s">
         <v>21</v>
       </c>
       <c r="J70" t="s">
@@ -3849,7 +3849,7 @@
       <c r="F71" t="s">
         <v>19</v>
       </c>
-      <c r="I71" t="s">
+      <c r="H71" t="s">
         <v>30</v>
       </c>
       <c r="K71" t="s">
@@ -3881,7 +3881,7 @@
       <c r="F72" t="s">
         <v>19</v>
       </c>
-      <c r="I72" t="s">
+      <c r="H72" t="s">
         <v>30</v>
       </c>
       <c r="J72" t="s">
@@ -3916,7 +3916,7 @@
       <c r="F73" t="s">
         <v>19</v>
       </c>
-      <c r="I73" t="s">
+      <c r="H73" t="s">
         <v>30</v>
       </c>
       <c r="J73" t="s">
@@ -3951,7 +3951,7 @@
       <c r="F74" t="s">
         <v>19</v>
       </c>
-      <c r="I74" t="s">
+      <c r="H74" t="s">
         <v>30</v>
       </c>
       <c r="K74" t="s">
@@ -3989,7 +3989,7 @@
       <c r="F75" t="s">
         <v>19</v>
       </c>
-      <c r="I75" t="s">
+      <c r="H75" t="s">
         <v>21</v>
       </c>
       <c r="J75" t="s">
@@ -4027,7 +4027,7 @@
       <c r="F76" t="s">
         <v>19</v>
       </c>
-      <c r="I76" t="s">
+      <c r="H76" t="s">
         <v>21</v>
       </c>
       <c r="J76" t="s">
@@ -4065,7 +4065,7 @@
       <c r="F77" t="s">
         <v>19</v>
       </c>
-      <c r="I77" t="s">
+      <c r="H77" t="s">
         <v>21</v>
       </c>
       <c r="J77" t="s">
@@ -4103,7 +4103,7 @@
       <c r="F78" t="s">
         <v>19</v>
       </c>
-      <c r="I78" t="s">
+      <c r="H78" t="s">
         <v>21</v>
       </c>
       <c r="J78" t="s">
@@ -4138,7 +4138,7 @@
       <c r="F79" t="s">
         <v>19</v>
       </c>
-      <c r="I79" t="s">
+      <c r="H79" t="s">
         <v>21</v>
       </c>
       <c r="K79" t="s">
@@ -4170,7 +4170,7 @@
       <c r="F80" t="s">
         <v>19</v>
       </c>
-      <c r="I80" t="s">
+      <c r="H80" t="s">
         <v>21</v>
       </c>
       <c r="K80" t="s">
@@ -4202,7 +4202,7 @@
       <c r="F81" t="s">
         <v>19</v>
       </c>
-      <c r="I81" t="s">
+      <c r="H81" t="s">
         <v>21</v>
       </c>
       <c r="K81" t="s">
@@ -4234,7 +4234,7 @@
       <c r="F82" t="s">
         <v>19</v>
       </c>
-      <c r="I82" t="s">
+      <c r="H82" t="s">
         <v>21</v>
       </c>
       <c r="K82" t="s">
@@ -4266,7 +4266,7 @@
       <c r="F83" t="s">
         <v>19</v>
       </c>
-      <c r="I83" t="s">
+      <c r="H83" t="s">
         <v>21</v>
       </c>
       <c r="J83" t="s">
@@ -4301,7 +4301,7 @@
       <c r="F84" t="s">
         <v>19</v>
       </c>
-      <c r="I84" t="s">
+      <c r="H84" t="s">
         <v>21</v>
       </c>
       <c r="K84" t="s">
@@ -4339,7 +4339,7 @@
       <c r="F85" t="s">
         <v>19</v>
       </c>
-      <c r="I85" t="s">
+      <c r="H85" t="s">
         <v>30</v>
       </c>
       <c r="J85" t="s">
@@ -4377,7 +4377,7 @@
       <c r="F86" t="s">
         <v>19</v>
       </c>
-      <c r="I86" t="s">
+      <c r="H86" t="s">
         <v>21</v>
       </c>
       <c r="J86" t="s">
@@ -4415,7 +4415,7 @@
       <c r="F87" t="s">
         <v>19</v>
       </c>
-      <c r="I87" t="s">
+      <c r="H87" t="s">
         <v>21</v>
       </c>
       <c r="J87" t="s">
@@ -4450,7 +4450,7 @@
       <c r="F88" t="s">
         <v>19</v>
       </c>
-      <c r="I88" t="s">
+      <c r="H88" t="s">
         <v>21</v>
       </c>
       <c r="J88" t="s">
@@ -4485,7 +4485,7 @@
       <c r="F89" t="s">
         <v>19</v>
       </c>
-      <c r="I89" t="s">
+      <c r="H89" t="s">
         <v>21</v>
       </c>
       <c r="J89" t="s">
@@ -4520,7 +4520,7 @@
       <c r="F90" t="s">
         <v>19</v>
       </c>
-      <c r="I90" t="s">
+      <c r="H90" t="s">
         <v>21</v>
       </c>
       <c r="J90" t="s">
@@ -4555,7 +4555,7 @@
       <c r="F91" t="s">
         <v>19</v>
       </c>
-      <c r="I91" t="s">
+      <c r="H91" t="s">
         <v>21</v>
       </c>
       <c r="J91" t="s">
@@ -4590,7 +4590,7 @@
       <c r="F92" t="s">
         <v>19</v>
       </c>
-      <c r="I92" t="s">
+      <c r="H92" t="s">
         <v>21</v>
       </c>
       <c r="J92" t="s">
@@ -4625,7 +4625,7 @@
       <c r="F93" t="s">
         <v>19</v>
       </c>
-      <c r="I93" t="s">
+      <c r="H93" t="s">
         <v>21</v>
       </c>
       <c r="J93" t="s">
@@ -4660,7 +4660,7 @@
       <c r="F94" t="s">
         <v>19</v>
       </c>
-      <c r="I94" t="s">
+      <c r="H94" t="s">
         <v>21</v>
       </c>
       <c r="J94" t="s">
@@ -4695,7 +4695,7 @@
       <c r="F95" t="s">
         <v>19</v>
       </c>
-      <c r="I95" t="s">
+      <c r="H95" t="s">
         <v>21</v>
       </c>
       <c r="J95" t="s">
@@ -4730,7 +4730,7 @@
       <c r="F96" t="s">
         <v>19</v>
       </c>
-      <c r="I96" t="s">
+      <c r="H96" t="s">
         <v>21</v>
       </c>
       <c r="J96" t="s">
@@ -4765,7 +4765,7 @@
       <c r="F97" t="s">
         <v>19</v>
       </c>
-      <c r="I97" t="s">
+      <c r="H97" t="s">
         <v>30</v>
       </c>
       <c r="K97" t="s">
@@ -4797,7 +4797,7 @@
       <c r="F98" t="s">
         <v>19</v>
       </c>
-      <c r="I98" t="s">
+      <c r="H98" t="s">
         <v>21</v>
       </c>
       <c r="K98" t="s">
@@ -4832,7 +4832,7 @@
       <c r="F99" t="s">
         <v>19</v>
       </c>
-      <c r="I99" t="s">
+      <c r="H99" t="s">
         <v>21</v>
       </c>
       <c r="K99" t="s">
@@ -4867,7 +4867,7 @@
       <c r="F100" t="s">
         <v>19</v>
       </c>
-      <c r="I100" t="s">
+      <c r="H100" t="s">
         <v>21</v>
       </c>
       <c r="K100" t="s">
@@ -4899,7 +4899,7 @@
       <c r="F101" t="s">
         <v>19</v>
       </c>
-      <c r="I101" t="s">
+      <c r="H101" t="s">
         <v>30</v>
       </c>
       <c r="J101" t="s">

</xml_diff>

<commit_message>
Completed merge all five files together -> Merge_ServiceWatch_Parameters
Next: Combine the shared SPN between the platforms.
</commit_message>
<xml_diff>
--- a/SWTest/Outputs/Finalists/DEET_Analysis_Final.xlsx
+++ b/SWTest/Outputs/Finalists/DEET_Analysis_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\Finalists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1966145-66EB-4886-8CBE-DFB4EB8E7BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0541B9-AC7B-4E7C-87A4-C44501AE1739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="4440" windowWidth="28455" windowHeight="8460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1308,14 +1308,14 @@
     <col min="4" max="5" width="6.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="59.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="59.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="34.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="222.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="143.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="57.85546875" style="2" customWidth="1"/>
+    <col min="15" max="15" width="46.7109375" style="2" customWidth="1"/>
     <col min="16" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
@@ -1342,10 +1342,10 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>9</v>
@@ -1388,7 +1388,7 @@
       <c r="G2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J2" s="3" t="s">
@@ -1414,7 +1414,7 @@
       <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -1446,7 +1446,7 @@
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>30</v>
       </c>
       <c r="L4" s="2" t="s">
@@ -1475,7 +1475,7 @@
       <c r="F5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J5" s="3" t="s">
@@ -1501,7 +1501,7 @@
       <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J6" s="3" t="s">
@@ -1527,7 +1527,7 @@
       <c r="F7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1553,7 +1553,7 @@
       <c r="F8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -1579,7 +1579,7 @@
       <c r="F9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J9" s="3" t="s">
@@ -1605,7 +1605,7 @@
       <c r="F10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J10" s="3" t="s">
@@ -1631,7 +1631,7 @@
       <c r="F11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J11" s="3" t="s">
@@ -1657,7 +1657,7 @@
       <c r="F12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J12" s="3" t="s">
@@ -1683,7 +1683,7 @@
       <c r="F13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J13" s="3" t="s">
@@ -1709,7 +1709,7 @@
       <c r="F14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J14" s="3" t="s">
@@ -1741,7 +1741,7 @@
       <c r="F15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J15" s="3" t="s">
@@ -1773,7 +1773,7 @@
       <c r="F16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J16" s="3" t="s">
@@ -1799,7 +1799,7 @@
       <c r="F17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J17" s="3" t="s">
@@ -1825,7 +1825,7 @@
       <c r="F18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J18" s="3" t="s">
@@ -1851,7 +1851,7 @@
       <c r="F19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>77</v>
       </c>
       <c r="J19" s="3" t="s">
@@ -1883,7 +1883,7 @@
       <c r="G20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J20" s="3" t="s">
@@ -1915,7 +1915,7 @@
       <c r="G21" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J21" s="3" t="s">
@@ -1950,7 +1950,7 @@
       <c r="G22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>77</v>
       </c>
       <c r="J22" s="3" t="s">
@@ -1985,7 +1985,7 @@
       <c r="G23" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       <c r="F24" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K24" s="2" t="s">
@@ -2040,7 +2040,7 @@
       <c r="F25" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K25" s="2" t="s">
@@ -2072,7 +2072,7 @@
       <c r="F26" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K26" s="2" t="s">
@@ -2104,7 +2104,7 @@
       <c r="F27" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K27" s="2" t="s">
@@ -2136,7 +2136,7 @@
       <c r="F28" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K28" s="2" t="s">
@@ -2168,7 +2168,7 @@
       <c r="F29" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I29" s="2" t="s">
+      <c r="H29" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J29" s="3" t="s">
@@ -2194,7 +2194,7 @@
       <c r="F30" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J30" s="3" t="s">
@@ -2220,7 +2220,7 @@
       <c r="F31" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J31" s="3" t="s">
@@ -2255,7 +2255,7 @@
       <c r="F32" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="H32" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J32" s="3" t="s">
@@ -2290,7 +2290,7 @@
       <c r="F33" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J33" s="3" t="s">
@@ -2316,7 +2316,7 @@
       <c r="F34" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="H34" s="2" t="s">
         <v>77</v>
       </c>
       <c r="J34" s="3" t="s">
@@ -2351,7 +2351,7 @@
       <c r="G35" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="H35" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J35" s="3" t="s">
@@ -2383,7 +2383,7 @@
       <c r="F36" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="H36" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J36" s="3" t="s">
@@ -2415,7 +2415,7 @@
       <c r="F37" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>21</v>
       </c>
       <c r="K37" s="4" t="b">
@@ -2447,7 +2447,7 @@
       <c r="G38" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J38" s="3" t="s">
@@ -2482,7 +2482,7 @@
       <c r="F39" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="H39" s="2" t="s">
         <v>30</v>
       </c>
       <c r="N39" s="2" t="s">
@@ -2511,7 +2511,7 @@
       <c r="F40" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J40" s="3" t="s">
@@ -2546,7 +2546,7 @@
       <c r="F41" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="H41" s="2" t="s">
         <v>21</v>
       </c>
       <c r="L41" s="2" t="s">
@@ -2575,7 +2575,7 @@
       <c r="F42" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="H42" s="2" t="s">
         <v>21</v>
       </c>
       <c r="L42" s="2" t="s">
@@ -2604,7 +2604,7 @@
       <c r="F43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="H43" s="2" t="s">
         <v>21</v>
       </c>
       <c r="L43" s="2" t="s">
@@ -2633,7 +2633,7 @@
       <c r="F44" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>21</v>
       </c>
       <c r="L44" s="2" t="s">
@@ -2662,7 +2662,7 @@
       <c r="F45" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
       <c r="F46" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       <c r="F47" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="H47" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       <c r="F48" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="H48" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       <c r="F49" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="H49" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       <c r="F50" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="H50" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J50" s="3" t="s">
@@ -2806,7 +2806,7 @@
       <c r="F51" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="H51" s="2" t="s">
         <v>21</v>
       </c>
       <c r="K51" s="2" t="s">
@@ -2858,7 +2858,7 @@
       <c r="F53" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="H53" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J53" s="3" t="s">
@@ -2884,7 +2884,7 @@
       <c r="F54" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I54" s="2" t="s">
+      <c r="H54" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2907,7 +2907,7 @@
       <c r="F55" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I55" s="2" t="s">
+      <c r="H55" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J55" s="3" t="s">
@@ -2933,7 +2933,7 @@
       <c r="F56" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I56" s="2" t="s">
+      <c r="H56" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J56" s="3" t="s">
@@ -2959,7 +2959,7 @@
       <c r="F57" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I57" s="2" t="s">
+      <c r="H57" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J57" s="3" t="s">
@@ -2985,7 +2985,7 @@
       <c r="F58" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I58" s="2" t="s">
+      <c r="H58" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J58" s="3" t="s">
@@ -3011,7 +3011,7 @@
       <c r="F59" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I59" s="2" t="s">
+      <c r="H59" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       <c r="F60" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I60" s="2" t="s">
+      <c r="H60" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J60" s="3" t="s">
@@ -3060,7 +3060,7 @@
       <c r="F61" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I61" s="2" t="s">
+      <c r="H61" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J61" s="3" t="s">
@@ -3086,7 +3086,7 @@
       <c r="F62" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I62" s="2" t="s">
+      <c r="H62" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J62" s="3" t="s">
@@ -3112,7 +3112,7 @@
       <c r="F63" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I63" s="2" t="s">
+      <c r="H63" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
       <c r="F64" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I64" s="2" t="s">
+      <c r="H64" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       <c r="F65" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I65" s="2" t="s">
+      <c r="H65" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       <c r="F66" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I66" s="2" t="s">
+      <c r="H66" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
       <c r="F67" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I67" s="2" t="s">
+      <c r="H67" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J67" s="3" t="s">
@@ -3230,7 +3230,7 @@
       <c r="F68" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I68" s="2" t="s">
+      <c r="H68" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J68" s="3" t="s">
@@ -3256,7 +3256,7 @@
       <c r="F69" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I69" s="2" t="s">
+      <c r="H69" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J69" s="3" t="s">
@@ -3282,7 +3282,7 @@
       <c r="F70" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I70" s="2" t="s">
+      <c r="H70" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J70" s="3" t="s">
@@ -3308,7 +3308,7 @@
       <c r="F71" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I71" s="2" t="s">
+      <c r="H71" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       <c r="F72" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I72" s="2" t="s">
+      <c r="H72" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J72" s="3" t="s">
@@ -3357,7 +3357,7 @@
       <c r="F73" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I73" s="2" t="s">
+      <c r="H73" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J73" s="3" t="s">
@@ -3383,7 +3383,7 @@
       <c r="F74" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I74" s="2" t="s">
+      <c r="H74" s="2" t="s">
         <v>30</v>
       </c>
       <c r="N74" s="2" t="s">
@@ -3412,7 +3412,7 @@
       <c r="F75" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I75" s="2" t="s">
+      <c r="H75" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J75" s="3" t="s">
@@ -3441,7 +3441,7 @@
       <c r="F76" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I76" s="2" t="s">
+      <c r="H76" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J76" s="3" t="s">
@@ -3470,7 +3470,7 @@
       <c r="F77" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I77" s="2" t="s">
+      <c r="H77" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J77" s="3" t="s">
@@ -3499,7 +3499,7 @@
       <c r="F78" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I78" s="2" t="s">
+      <c r="H78" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J78" s="3" t="s">
@@ -3525,7 +3525,7 @@
       <c r="F79" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I79" s="2" t="s">
+      <c r="H79" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       <c r="F80" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I80" s="2" t="s">
+      <c r="H80" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       <c r="F81" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I81" s="2" t="s">
+      <c r="H81" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       <c r="F82" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I82" s="2" t="s">
+      <c r="H82" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3617,7 +3617,7 @@
       <c r="F83" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I83" s="2" t="s">
+      <c r="H83" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J83" s="3" t="s">
@@ -3643,7 +3643,7 @@
       <c r="F84" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I84" s="2" t="s">
+      <c r="H84" s="2" t="s">
         <v>21</v>
       </c>
       <c r="K84" s="2" t="s">
@@ -3675,7 +3675,7 @@
       <c r="F85" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I85" s="2" t="s">
+      <c r="H85" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J85" s="3" t="s">
@@ -3707,7 +3707,7 @@
       <c r="F86" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I86" s="2" t="s">
+      <c r="H86" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J86" s="3" t="s">
@@ -3736,7 +3736,7 @@
       <c r="F87" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I87" s="2" t="s">
+      <c r="H87" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J87" s="3" t="s">
@@ -3762,7 +3762,7 @@
       <c r="F88" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I88" s="2" t="s">
+      <c r="H88" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J88" s="3" t="s">
@@ -3788,7 +3788,7 @@
       <c r="F89" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I89" s="2" t="s">
+      <c r="H89" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J89" s="3" t="s">
@@ -3814,7 +3814,7 @@
       <c r="F90" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I90" s="2" t="s">
+      <c r="H90" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J90" s="3" t="s">
@@ -3840,7 +3840,7 @@
       <c r="F91" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I91" s="2" t="s">
+      <c r="H91" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J91" s="3" t="s">
@@ -3866,7 +3866,7 @@
       <c r="F92" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I92" s="2" t="s">
+      <c r="H92" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J92" s="3" t="s">
@@ -3892,7 +3892,7 @@
       <c r="F93" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I93" s="2" t="s">
+      <c r="H93" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J93" s="3" t="s">
@@ -3918,7 +3918,7 @@
       <c r="F94" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I94" s="2" t="s">
+      <c r="H94" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J94" s="3" t="s">
@@ -3944,7 +3944,7 @@
       <c r="F95" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I95" s="2" t="s">
+      <c r="H95" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J95" s="3" t="s">
@@ -3970,7 +3970,7 @@
       <c r="F96" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I96" s="2" t="s">
+      <c r="H96" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J96" s="3" t="s">
@@ -3996,7 +3996,7 @@
       <c r="F97" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I97" s="2" t="s">
+      <c r="H97" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -4019,7 +4019,7 @@
       <c r="F98" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I98" s="2" t="s">
+      <c r="H98" s="2" t="s">
         <v>21</v>
       </c>
       <c r="N98" s="2" t="s">
@@ -4045,7 +4045,7 @@
       <c r="F99" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I99" s="2" t="s">
+      <c r="H99" s="2" t="s">
         <v>21</v>
       </c>
       <c r="N99" s="2" t="s">
@@ -4071,7 +4071,7 @@
       <c r="F100" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I100" s="2" t="s">
+      <c r="H100" s="2" t="s">
         <v>21</v>
       </c>
       <c r="N100" s="2" t="s">
@@ -4094,7 +4094,7 @@
       <c r="F101" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I101" s="2" t="s">
+      <c r="H101" s="2" t="s">
         <v>30</v>
       </c>
       <c r="J101" s="3" t="s">

</xml_diff>